<commit_message>
Remove Comments and Rerun Exec
</commit_message>
<xml_diff>
--- a/excel/assoc/out.xlsx
+++ b/excel/assoc/out.xlsx
@@ -1852,7 +1852,7 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Articulated</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Articulated</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">

</xml_diff>